<commit_message>
UPDATE: Random & OfYourChoice Icon updated
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CDE9714-5FAD-44B1-A04B-8AC3BF35C9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674F6020-D61D-4FA1-B4A8-37D749371868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
   <si>
     <t>en</t>
   </si>
@@ -864,6 +864,18 @@
   </si>
   <si>
     <t>TRADE_TITLE</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>ORANGE</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Orange</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>橘子</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1832,7 +1844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36.75" customWidth="1"/>
@@ -1996,705 +2008,716 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>3</v>
+        <v>234</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>114</v>
+        <v>235</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>195</v>
+        <v>119</v>
       </c>
       <c r="C22" t="s">
-        <v>196</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>121</v>
+        <v>195</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>197</v>
+        <v>122</v>
       </c>
       <c r="C25" t="s">
-        <v>198</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C26" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>125</v>
+        <v>199</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C28" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>138</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C33" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C34" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>141</v>
-      </c>
-      <c r="B36" t="s">
-        <v>170</v>
+        <v>140</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>174</v>
       </c>
       <c r="C36" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>142</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>172</v>
+        <v>141</v>
+      </c>
+      <c r="B37" t="s">
+        <v>170</v>
       </c>
       <c r="C37" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
+        <v>142</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C38" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
         <v>143</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A39" t="s">
+    <row r="40" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A40" t="s">
         <v>144</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C40" t="s">
         <v>166</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>145</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="C40" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C41" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C42" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C43" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="C44" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>190</v>
+        <v>204</v>
       </c>
       <c r="C45" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C46" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C47" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C49" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>221</v>
+        <v>183</v>
       </c>
       <c r="C50" t="s">
-        <v>222</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>184</v>
+        <v>221</v>
       </c>
       <c r="C51" t="s">
-        <v>160</v>
+        <v>222</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>156</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C52" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
         <v>157</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B53" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C53" t="s">
         <v>161</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>214</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C55" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C56" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>19</v>
+        <v>209</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>20</v>
+        <v>210</v>
       </c>
       <c r="C57" t="s">
-        <v>71</v>
+        <v>211</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C58" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C59" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C60" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C61" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C62" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C63" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C64" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
+        <v>35</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" t="s">
         <v>37</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B67" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C66" t="s">
+      <c r="C67" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A67" t="s">
-        <v>39</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C67" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="14.25" customHeight="1">
       <c r="A68" t="s">
-        <v>108</v>
+        <v>39</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>109</v>
+        <v>40</v>
       </c>
       <c r="C68" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="14.25" customHeight="1">
       <c r="A69" t="s">
+        <v>108</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C69" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A70" t="s">
         <v>111</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B70" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C70" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
-      <c r="A71" t="s">
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
         <v>41</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B72" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C72" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="28.5">
-      <c r="A72" t="s">
+    <row r="73" spans="1:3" ht="28.5">
+      <c r="A73" t="s">
         <v>42</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B73" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C73" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
-      <c r="A73" t="s">
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
         <v>43</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B74" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C74" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="28.5">
-      <c r="A74" t="s">
+    <row r="75" spans="1:3" ht="28.5">
+      <c r="A75" t="s">
         <v>44</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B75" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C74" s="1" t="s">
+      <c r="C75" s="1" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>45</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
+        <v>53</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
         <v>55</v>
       </c>
-      <c r="B80" s="2" t="s">
+      <c r="B81" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C81" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="28.5">
-      <c r="A81" t="s">
+    <row r="82" spans="1:3" ht="28.5">
+      <c r="A82" t="s">
         <v>56</v>
       </c>
-      <c r="B81" s="1" t="s">
+      <c r="B82" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C82" s="1" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82" t="s">
-        <v>215</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
+        <v>215</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" t="s">
         <v>216</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="B84" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C84" t="s">
         <v>217</v>
       </c>
     </row>

</xml_diff>

<commit_message>
UPDATE: NEW upgrade added
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674F6020-D61D-4FA1-B4A8-37D749371868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B965352E-3F02-4118-909E-53BDA87B56CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-7310" windowWidth="21820" windowHeight="37900" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
   <sheets>
     <sheet name="String_Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="243">
   <si>
     <t>en</t>
   </si>
@@ -876,6 +876,28 @@
   </si>
   <si>
     <t>橘子</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>LOTTERY_REMOTE_DRAW</t>
+  </si>
+  <si>
+    <t>lottery remote draw</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>远程抽奖</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>LOTTERY_REMOTE_DRAW_DESCRIPTION</t>
+  </si>
+  <si>
+    <t>抽奖券现在可以远程进行水果抽奖。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Draw Coupon now can be used to draw remotely.</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1844,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36.75" customWidth="1"/>
@@ -2413,6 +2435,17 @@
         <v>161</v>
       </c>
     </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>237</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C55" t="s">
+        <v>239</v>
+      </c>
+    </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
         <v>214</v>
@@ -2719,6 +2752,17 @@
       </c>
       <c r="C84" t="s">
         <v>217</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" t="s">
+        <v>240</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C85" t="s">
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Hours become Minutes
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4A9074-F9D7-487C-90A4-92956864BA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{900C5CD4-7FDB-4B5A-94AB-1E8598240888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -223,12 +223,6 @@
     <t>key</t>
   </si>
   <si>
-    <t>DAY %s\n%s:00\n[font_size=26]Shop refresh in %sh[/font_size]</t>
-  </si>
-  <si>
-    <t>第 %s 天\n%s:00\n[font_size=26]商店将在 %s 小时后刷新[/font_size]</t>
-  </si>
-  <si>
     <t>事务升级券</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -573,6 +567,14 @@
   </si>
   <si>
     <t>Yellow</t>
+  </si>
+  <si>
+    <t>%02d:%02d\n[font_size=26]Shop refresh in %smin[/font_size]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>%02d:%02d\n[font_size=26]商店将在 %s 分钟后刷新[/font_size]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1554,43 +1556,43 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>67</v>
+        <v>160</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" t="s">
         <v>122</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" t="s">
         <v>125</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C4" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" t="s">
         <v>126</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C5" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1598,10 +1600,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1609,10 +1611,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1620,10 +1622,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1631,10 +1633,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1642,10 +1644,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1653,10 +1655,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1664,10 +1666,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1675,10 +1677,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1686,10 +1688,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1697,10 +1699,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1708,10 +1710,10 @@
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1719,10 +1721,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1730,10 +1732,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1741,10 +1743,10 @@
         <v>16</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C20" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1752,10 +1754,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1763,10 +1765,10 @@
         <v>18</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1774,10 +1776,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1785,10 +1787,10 @@
         <v>20</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1796,10 +1798,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1807,10 +1809,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C26" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1818,10 +1820,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1829,10 +1831,10 @@
         <v>24</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1840,10 +1842,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1851,10 +1853,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C30" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1862,10 +1864,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C31" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1876,7 +1878,7 @@
         <v>29</v>
       </c>
       <c r="C33" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1887,7 +1889,7 @@
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1898,7 +1900,7 @@
         <v>33</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1909,7 +1911,7 @@
         <v>35</v>
       </c>
       <c r="C36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1920,7 +1922,7 @@
         <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1931,7 +1933,7 @@
         <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1942,7 +1944,7 @@
         <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1953,7 +1955,7 @@
         <v>43</v>
       </c>
       <c r="C40" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1964,7 +1966,7 @@
         <v>45</v>
       </c>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1975,7 +1977,7 @@
         <v>47</v>
       </c>
       <c r="C42" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1">
@@ -1986,29 +1988,29 @@
         <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" t="s">
+        <v>129</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C44" t="s">
         <v>131</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C44" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>132</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="C45" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -2016,10 +2018,10 @@
         <v>50</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="28.5">
@@ -2027,10 +2029,10 @@
         <v>51</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -2038,10 +2040,10 @@
         <v>52</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="28.5">
@@ -2049,10 +2051,10 @@
         <v>53</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -2063,7 +2065,7 @@
         <v>55</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -2074,7 +2076,7 @@
         <v>57</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -2085,7 +2087,7 @@
         <v>59</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -2096,7 +2098,7 @@
         <v>61</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -2107,7 +2109,7 @@
         <v>63</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -2115,10 +2117,10 @@
         <v>64</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="28.5">
@@ -2126,10 +2128,10 @@
         <v>65</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: Bunch of updates from PoC_off_work except for balls
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364D408A-ABFA-40EA-92A4-5929CBEB7587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE6CAE6-9A0B-43D2-9492-E9CEC91282AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="245">
   <si>
     <t>en</t>
   </si>
@@ -475,22 +475,6 @@
   </si>
   <si>
     <t>TIME_REFRESH</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>TIME_DAY_HOUR</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>[font_size=26]商店将在 %s 小时后刷新[/font_size]</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>[font_size=26]Shop refresh in %sh[/font_size]</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>第 %s 天\n%02d:00\n</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
@@ -751,9 +735,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>DAY %s\n%02d:00\n</t>
-  </si>
-  <si>
     <t>%.1f%%\n[font_size=34]SUCCESS RATE[/font_size]</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -898,6 +879,34 @@
   </si>
   <si>
     <t>Once left, you will not be able to return.\nAre you sure to start the adventure?</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>TIME_DAY_HOUR_MINUTE</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>DAY %s\n%02d:%02d\n</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>第 %s 天\n%02d:%02d\n</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[font_size=26]商店将在 %s 分钟后刷新[/font_size]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[font_size=26]Shop refresh in %smin[/font_size]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOLD</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>售罄</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1866,7 +1875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36.75" customWidth="1"/>
@@ -1887,13 +1896,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>238</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>204</v>
+        <v>239</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1901,560 +1910,560 @@
         <v>131</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>134</v>
+        <v>242</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C4" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>99</v>
+        <v>243</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>100</v>
+        <v>243</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>223</v>
+        <v>125</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>222</v>
+        <v>129</v>
       </c>
       <c r="C9" t="s">
-        <v>221</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C13" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C15" t="s">
-        <v>200</v>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>226</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>232</v>
+        <v>2</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>233</v>
+        <v>195</v>
       </c>
       <c r="C16" t="s">
-        <v>234</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>227</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>112</v>
+        <v>228</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>193</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>194</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>119</v>
+        <v>189</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>195</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>196</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C27" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>123</v>
+        <v>193</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C32" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
         <v>9</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C33" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>136</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C34" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C35" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C36" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>139</v>
-      </c>
-      <c r="B37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>168</v>
       </c>
       <c r="C37" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>140</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>170</v>
+        <v>135</v>
+      </c>
+      <c r="B38" t="s">
+        <v>164</v>
       </c>
       <c r="C38" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="C39" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>137</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A41" t="s">
+        <v>138</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C41" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A40" t="s">
-        <v>142</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="C40" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>143</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C41" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C42" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C43" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C44" t="s">
-        <v>184</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="C45" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="C46" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C47" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C48" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C49" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" t="s">
         <v>152</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="C50" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
+        <v>148</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C51" t="s">
         <v>153</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C51" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>182</v>
+        <v>214</v>
       </c>
       <c r="C52" t="s">
-        <v>158</v>
+        <v>215</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>150</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="C53" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
+        <v>151</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C54" t="s">
         <v>155</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="C53" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
-      <c r="A55" t="s">
-        <v>235</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C55" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="C56" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -2462,307 +2471,318 @@
         <v>207</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C57" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>19</v>
+        <v>202</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>20</v>
+        <v>203</v>
       </c>
       <c r="C58" t="s">
-        <v>71</v>
+        <v>204</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C59" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C60" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C61" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C62" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C63" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C64" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C65" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C66" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
+        <v>35</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C67" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" t="s">
         <v>37</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B68" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C68" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A68" t="s">
-        <v>39</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C68" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="14.25" customHeight="1">
       <c r="A69" t="s">
-        <v>108</v>
+        <v>39</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>109</v>
+        <v>40</v>
       </c>
       <c r="C69" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="14.25" customHeight="1">
       <c r="A70" t="s">
+        <v>108</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C70" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A71" t="s">
         <v>111</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="C70" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3">
-      <c r="A72" t="s">
+      <c r="B71" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C71" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
         <v>41</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B73" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C73" s="2" t="s">
         <v>86</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="28.5">
-      <c r="A73" t="s">
-        <v>42</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
+        <v>42</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
         <v>43</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B75" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C75" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="28.5">
-      <c r="A75" t="s">
+    <row r="76" spans="1:3" ht="28.5">
+      <c r="A76" t="s">
         <v>44</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B76" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C76" s="1" t="s">
         <v>90</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76" t="s">
-        <v>45</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
+        <v>53</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" t="s">
         <v>55</v>
       </c>
-      <c r="B81" s="2" t="s">
+      <c r="B82" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C82" s="2" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="28.5">
-      <c r="A82" t="s">
-        <v>56</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>213</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="C83" s="3" t="s">
-        <v>217</v>
+        <v>56</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>214</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="C84" t="s">
-        <v>215</v>
+        <v>208</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>238</v>
+        <v>209</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
       <c r="C85" t="s">
-        <v>239</v>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" t="s">
+        <v>233</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C86" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: 3 Types of MBox n PrizeSource added; itemforsale Count added; Shop nonrepeat n 3choose1
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE6CAE6-9A0B-43D2-9492-E9CEC91282AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8586CC-B40F-4B37-82C8-B11C573FBFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
+    <workbookView xWindow="15480" yWindow="1095" windowWidth="21780" windowHeight="20985" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
   <sheets>
     <sheet name="String_Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="251">
   <si>
     <t>en</t>
   </si>
@@ -228,10 +228,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>盲盒</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>商店刷新</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -436,9 +432,6 @@
   </si>
   <si>
     <t>Mystery Box</t>
-  </si>
-  <si>
-    <t>Shop Refresh</t>
   </si>
   <si>
     <t>Strawberry</t>
@@ -908,6 +901,36 @@
   <si>
     <t>售罄</t>
     <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>大盲盒</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shop Refresh</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>UPGRADE_COUPON_MYSTERY_BOX</t>
+  </si>
+  <si>
+    <t>Upgrade Coupon Mystery Box</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>升级券盲盒</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>物资盲盒</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Supply Mystery Box</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>SUPPLY_MYSTERY_BOX</t>
   </si>
 </sst>
 </file>
@@ -1875,7 +1898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36.75" customWidth="1"/>
@@ -1896,145 +1919,145 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>236</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C2" t="s">
         <v>238</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="C2" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" t="s">
         <v>199</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C4" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" t="s">
         <v>100</v>
-      </c>
-      <c r="C6" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C14" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -2042,21 +2065,21 @@
         <v>2</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C16" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>225</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C17" t="s">
         <v>227</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C17" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -2064,7 +2087,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
         <v>58</v>
@@ -2075,7 +2098,7 @@
         <v>4</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -2086,7 +2109,7 @@
         <v>5</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C20" t="s">
         <v>60</v>
@@ -2097,7 +2120,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C21" t="s">
         <v>61</v>
@@ -2108,7 +2131,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C22" t="s">
         <v>62</v>
@@ -2119,7 +2142,7 @@
         <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
         <v>63</v>
@@ -2130,10 +2153,10 @@
         <v>10</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C24" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -2141,7 +2164,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C25" t="s">
         <v>65</v>
@@ -2152,10 +2175,10 @@
         <v>12</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -2163,10 +2186,10 @@
         <v>15</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C27" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2174,10 +2197,10 @@
         <v>16</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C28" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2185,10 +2208,10 @@
         <v>17</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2196,10 +2219,10 @@
         <v>13</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>121</v>
+        <v>244</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2207,10 +2230,10 @@
         <v>14</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2218,10 +2241,10 @@
         <v>18</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2229,106 +2252,106 @@
         <v>9</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C33" t="s">
         <v>64</v>
       </c>
     </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>250</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C34" t="s">
+        <v>248</v>
+      </c>
+    </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>132</v>
+        <v>245</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>170</v>
+        <v>246</v>
       </c>
       <c r="C35" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>133</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="C36" t="s">
-        <v>163</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>168</v>
       </c>
       <c r="C37" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>135</v>
-      </c>
-      <c r="B38" t="s">
-        <v>164</v>
+        <v>131</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>167</v>
       </c>
       <c r="C38" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>166</v>
       </c>
       <c r="C39" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>137</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>171</v>
+        <v>133</v>
+      </c>
+      <c r="B40" t="s">
+        <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="13.5" customHeight="1">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="C41" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C42" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="13.5" customHeight="1">
       <c r="A43" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C43" t="s">
         <v>158</v>
@@ -2336,453 +2359,475 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C45" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="C46" t="s">
-        <v>197</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C47" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="C48" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C49" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C50" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="C51" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>214</v>
+        <v>174</v>
       </c>
       <c r="C52" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C53" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>179</v>
+        <v>212</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>148</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C55" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>230</v>
+        <v>149</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="C56" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" t="s">
-        <v>207</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C57" t="s">
-        <v>206</v>
+        <v>153</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>202</v>
+        <v>228</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
       <c r="C58" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>19</v>
+        <v>205</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>20</v>
+        <v>203</v>
       </c>
       <c r="C59" t="s">
-        <v>71</v>
+        <v>204</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>21</v>
+        <v>200</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>22</v>
+        <v>201</v>
       </c>
       <c r="C60" t="s">
-        <v>72</v>
+        <v>202</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C61" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C62" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C63" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C64" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C65" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C66" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C67" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>33</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C68" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>35</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C69" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
         <v>37</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B70" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C68" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A69" t="s">
-        <v>39</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C69" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A70" t="s">
-        <v>108</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>109</v>
-      </c>
       <c r="C70" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="14.25" customHeight="1">
       <c r="A71" t="s">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>237</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A72" t="s">
+        <v>107</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C72" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="14.25" customHeight="1">
       <c r="A73" t="s">
-        <v>41</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3">
-      <c r="A74" t="s">
-        <v>42</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>87</v>
+        <v>110</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C73" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="28.5">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>44</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>90</v>
+        <v>42</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>45</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
+        <v>43</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="28.5">
       <c r="A78" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>55</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>96</v>
+        <v>51</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>97</v>
+        <v>54</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>208</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>212</v>
+        <v>55</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>209</v>
+        <v>56</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C85" t="s">
-        <v>210</v>
+        <v>96</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
+        <v>206</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C86" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" t="s">
+        <v>207</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C87" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>231</v>
+      </c>
+      <c r="B88" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B86" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="C86" t="s">
-        <v>234</v>
+      <c r="C88" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UPDATE: shop panel text added; grande Mbox icon changed
</commit_message>
<xml_diff>
--- a/Assets/Internationalization/String_Data.xlsx
+++ b/Assets/Internationalization/String_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Game Projects\Godot Projects\city_of_circling\Assets\Internationalization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8586CC-B40F-4B37-82C8-B11C573FBFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92398486-9A8C-4894-B079-2171F1DDE9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15480" yWindow="1095" windowWidth="21780" windowHeight="20985" xr2:uid="{08590711-CB36-410F-B5A8-7B8F5AA8D814}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="254">
   <si>
     <t>en</t>
   </si>
@@ -931,6 +931,17 @@
   </si>
   <si>
     <t>SUPPLY_MYSTERY_BOX</t>
+  </si>
+  <si>
+    <t>PICK_1_OF_3</t>
+  </si>
+  <si>
+    <t>选择一项购买</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pick 1 Of 3 To Purchase</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1898,7 +1909,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D1D195-E5E8-4810-8E47-E25327235024}">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="36.75" customWidth="1"/>
@@ -1974,859 +1985,870 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>251</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>106</v>
+        <v>253</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>123</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>215</v>
+        <v>127</v>
       </c>
       <c r="C10" t="s">
-        <v>214</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C11" t="s">
-        <v>124</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C14" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
         <v>224</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="C16" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>225</v>
+        <v>2</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>226</v>
+        <v>193</v>
       </c>
       <c r="C17" t="s">
-        <v>227</v>
+        <v>194</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>225</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>111</v>
+        <v>226</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>187</v>
+        <v>116</v>
       </c>
       <c r="C24" t="s">
-        <v>188</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>118</v>
+        <v>187</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>188</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C26" t="s">
-        <v>243</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>189</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>190</v>
+        <v>243</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C28" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>121</v>
+        <v>191</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>192</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>244</v>
+        <v>121</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>120</v>
+        <v>244</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>250</v>
+        <v>9</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>249</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
-        <v>248</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
+        <v>250</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C35" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
         <v>245</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C36" t="s">
         <v>247</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>130</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C37" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C38" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C39" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>133</v>
-      </c>
-      <c r="B40" t="s">
-        <v>162</v>
+        <v>132</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="C40" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>134</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>164</v>
+        <v>133</v>
+      </c>
+      <c r="B41" t="s">
+        <v>162</v>
       </c>
       <c r="C41" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>134</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C42" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
         <v>135</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C43" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A43" t="s">
+    <row r="44" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A44" t="s">
         <v>136</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C44" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>137</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C44" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C45" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C46" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C47" t="s">
-        <v>178</v>
+        <v>157</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="C48" t="s">
-        <v>195</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>182</v>
+        <v>196</v>
       </c>
       <c r="C49" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C50" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C51" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="C52" t="s">
-        <v>150</v>
+        <v>185</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>212</v>
+        <v>175</v>
       </c>
       <c r="C54" t="s">
-        <v>213</v>
+        <v>151</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>176</v>
+        <v>212</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>213</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>148</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C56" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>149</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B57" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>153</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>228</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="C58" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>205</v>
+        <v>228</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
       <c r="C59" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C60" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>19</v>
+        <v>200</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>20</v>
+        <v>201</v>
       </c>
       <c r="C61" t="s">
-        <v>70</v>
+        <v>202</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C63" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C64" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C66" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C67" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C68" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C69" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>35</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C70" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
         <v>37</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B71" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C71" t="s">
         <v>79</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A71" t="s">
-        <v>39</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C71" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="14.25" customHeight="1">
       <c r="A72" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="C72" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="14.25" customHeight="1">
       <c r="A73" t="s">
+        <v>107</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C73" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A74" t="s">
         <v>110</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B74" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C74" t="s">
         <v>234</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>41</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
+        <v>42</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
         <v>43</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B78" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C78" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="28.5">
-      <c r="A78" t="s">
+    <row r="79" spans="1:3" ht="28.5">
+      <c r="A79" t="s">
         <v>44</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B79" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C79" s="1" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3">
-      <c r="A79" t="s">
-        <v>45</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>55</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>95</v>
+        <v>53</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>56</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>97</v>
+        <v>55</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>206</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>210</v>
+        <v>56</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>207</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C87" t="s">
-        <v>208</v>
+        <v>206</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
+        <v>207</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C88" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" t="s">
         <v>231</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="B89" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C89" t="s">
         <v>232</v>
       </c>
     </row>

</xml_diff>